<commit_message>
informe mensual septiembre 2023
informe mensual septiembre 2023 - OK
</commit_message>
<xml_diff>
--- a/tools/AMH Sedes BC.xlsx
+++ b/tools/AMH Sedes BC.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive - CELSIA S.A E.S.P\Extralaboral\Mensual\push_20221130\tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://celsia-my.sharepoint.com/personal/jpocampo_celsia_com/Documents/ESCRITORIO_2023/bc_mensual/CB_Informe_Mensual/tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A447CF0C-7C99-4CB6-8A65-DFA915F8A16C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A447CF0C-7C99-4CB6-8A65-DFA915F8A16C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75B6821E-21EA-4F7D-88CE-E8BDA7C6B2DD}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="19965" windowHeight="21000" xr2:uid="{F5BB8399-9314-47A2-B594-4E7B5E3E1792}"/>
-    <workbookView xWindow="390" yWindow="390" windowWidth="19965" windowHeight="21000" xr2:uid="{654318A1-CC56-4612-872C-39964BF74505}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5BB8399-9314-47A2-B594-4E7B5E3E1792}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{654318A1-CC56-4612-872C-39964BF74505}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$J$65</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2187,7 +2187,6 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C2EFBC7-4BE6-4923-857D-D71BB095632F}" name="Table1" displayName="Table1" ref="A1:K1048576" totalsRowShown="0">
-  <autoFilter ref="A1:K1048576" xr:uid="{0C2EFBC7-4BE6-4923-857D-D71BB095632F}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K65">
     <sortCondition ref="A1:A1048576"/>
   </sortState>
@@ -2209,7 +2208,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2506,7 +2505,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5089703-7751-4A9C-AC83-25A9278D4BE1}">
   <dimension ref="A1:K65"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.42578125" style="6" bestFit="1" customWidth="1"/>
@@ -4655,7 +4654,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FFC24B4-2A7C-4DA8-B9F1-D0EE7B71ED02}">
   <dimension ref="A1:B520"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>

</xml_diff>